<commit_message>
Add "Incubated at 37C" as preparation_condition
Closes #148
</commit_message>
<xml_diff>
--- a/sample-section/latest/sample-section.xlsx
+++ b/sample-section/latest/sample-section.xlsx
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="171">
   <si>
     <t>source_id</t>
   </si>
@@ -380,30 +380,30 @@
     <t>http://purl.bioontology.org/ontology/MESH/C046311</t>
   </si>
   <si>
-    <t>UW Solution</t>
+    <t>MACS tissue storage solution</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000105</t>
+  </si>
+  <si>
+    <t>Fresh frozen CMC</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000130</t>
+  </si>
+  <si>
+    <t>Fresh frozen gelatin</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000198</t>
+  </si>
+  <si>
+    <t>UWS Solution</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000151</t>
   </si>
   <si>
-    <t>MACS tissue storage solution</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000105</t>
-  </si>
-  <si>
-    <t>Fresh frozen CMC</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000130</t>
-  </si>
-  <si>
-    <t>Fresh frozen gelatin</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000198</t>
-  </si>
-  <si>
     <t>Growth media</t>
   </si>
   <si>
@@ -473,6 +473,12 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185338</t>
   </si>
   <si>
+    <t>Incubated at 37 degrees celsius</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
+  </si>
+  <si>
     <t>Frozen at -20 degrees celsius</t>
   </si>
   <si>
@@ -542,6 +548,12 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C83594</t>
   </si>
   <si>
+    <t>Nuclease-free water</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000482</t>
+  </si>
+  <si>
     <t>1X quench buffer</t>
   </si>
   <si>
@@ -587,12 +599,6 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000387</t>
   </si>
   <si>
-    <t>Incubated at 37 degrees celsius</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
-  </si>
-  <si>
     <t>Frozen at -80 degrees celsius</t>
   </si>
   <si>
@@ -683,7 +689,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2025-11-03T17:31:25-08:00</t>
+    <t>2026-03-03T15:12:29-08:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -832,51 +838,51 @@
         <v>87</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="M1" t="s" s="1">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="N1" t="s" s="1">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="V1" t="s" s="1">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2">
       <c r="V2" t="s" s="23">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +898,7 @@
       <formula1>'preparation_medium'!$A$1:$A$35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_condition'!$A$1:$A$9</formula1>
+      <formula1>'preparation_condition'!$A$1:$A$10</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
@@ -902,7 +908,7 @@
       <formula1>'processing_time_unit'!$A$1:$A$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'storage_medium'!$A$1:$A$25</formula1>
+      <formula1>'storage_medium'!$A$1:$A$26</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="L2:L1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'storage_method'!$A$1:$A$12</formula1>
@@ -942,12 +948,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -968,30 +974,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1341,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1414,6 +1420,14 @@
       </c>
       <c r="B9" t="s" s="0">
         <v>103</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1457,23 +1471,23 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -1494,10 +1508,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -1518,145 +1532,153 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>46</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>119</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>120</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>55</v>
+        <v>123</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>56</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>122</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>59</v>
+        <v>125</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>60</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>124</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>75</v>
+        <v>131</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>76</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>130</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B26" t="s" s="0">
         <v>82</v>
       </c>
     </row>
@@ -1712,50 +1734,50 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>134</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>135</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12">
@@ -1778,26 +1800,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1812,18 +1834,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>